<commit_message>
Uprosc do plaskiego skryptu w komorkach (#%%), modele budowane wprost
</commit_message>
<xml_diff>
--- a/outputs/wyniki_regresji.xlsx
+++ b/outputs/wyniki_regresji.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,40 +442,35 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Srednia</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Srednia</t>
+          <t>Odch. std.</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Odch. std.</t>
+          <t>Min</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Min</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Max</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Max</t>
+          <t>Skosnosc</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Skosnosc</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Kurtoza</t>
         </is>
@@ -488,27 +483,24 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>251.42</v>
       </c>
       <c r="C2" t="n">
-        <v>251.42</v>
+        <v>263.4</v>
       </c>
       <c r="D2" t="n">
-        <v>263.4</v>
+        <v>31</v>
       </c>
       <c r="E2" t="n">
-        <v>31</v>
+        <v>113.5</v>
       </c>
       <c r="F2" t="n">
-        <v>113.5</v>
+        <v>824</v>
       </c>
       <c r="G2" t="n">
-        <v>824</v>
+        <v>1.164</v>
       </c>
       <c r="H2" t="n">
-        <v>1.164</v>
-      </c>
-      <c r="I2" t="n">
         <v>0.241</v>
       </c>
     </row>
@@ -519,27 +511,24 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12</v>
+        <v>96.42</v>
       </c>
       <c r="C3" t="n">
-        <v>96.42</v>
+        <v>45.94</v>
       </c>
       <c r="D3" t="n">
-        <v>45.94</v>
+        <v>55.8</v>
       </c>
       <c r="E3" t="n">
-        <v>55.8</v>
+        <v>66.02</v>
       </c>
       <c r="F3" t="n">
-        <v>66.02</v>
+        <v>174.02</v>
       </c>
       <c r="G3" t="n">
-        <v>174.02</v>
+        <v>0.612</v>
       </c>
       <c r="H3" t="n">
-        <v>0.612</v>
-      </c>
-      <c r="I3" t="n">
         <v>-1.573</v>
       </c>
     </row>
@@ -550,27 +539,24 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>383.5</v>
       </c>
       <c r="C4" t="n">
-        <v>383.5</v>
+        <v>116.29</v>
       </c>
       <c r="D4" t="n">
-        <v>116.29</v>
+        <v>233.31</v>
       </c>
       <c r="E4" t="n">
-        <v>233.31</v>
+        <v>374.83</v>
       </c>
       <c r="F4" t="n">
-        <v>374.83</v>
+        <v>541.92</v>
       </c>
       <c r="G4" t="n">
-        <v>541.92</v>
+        <v>-0.041</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.041</v>
-      </c>
-      <c r="I4" t="n">
         <v>-1.605</v>
       </c>
     </row>
@@ -581,27 +567,24 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12</v>
+        <v>-46.56</v>
       </c>
       <c r="C5" t="n">
-        <v>-46.56</v>
+        <v>64.42</v>
       </c>
       <c r="D5" t="n">
-        <v>64.42</v>
+        <v>-155.6</v>
       </c>
       <c r="E5" t="n">
-        <v>-155.6</v>
+        <v>-26.15</v>
       </c>
       <c r="F5" t="n">
-        <v>-26.15</v>
+        <v>42.46</v>
       </c>
       <c r="G5" t="n">
-        <v>42.46</v>
+        <v>-0.503</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.503</v>
-      </c>
-      <c r="I5" t="n">
         <v>-0.729</v>
       </c>
     </row>
@@ -612,27 +595,24 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12</v>
+        <v>0.25</v>
       </c>
       <c r="C6" t="n">
-        <v>0.25</v>
+        <v>0.45</v>
       </c>
       <c r="D6" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>1.327</v>
       </c>
       <c r="H6" t="n">
-        <v>1.327</v>
-      </c>
-      <c r="I6" t="n">
         <v>-0.326</v>
       </c>
     </row>

</xml_diff>